<commit_message>
Confirm actually-accomplished tasks in tracker, independent of scheduled date
- Row 2 (2026-08-24, Confirm Phase 0 decisions): Done -- locked
  constraints were cross-checked against the roadmap this session
- Row 4 (2026-08-26, Scaffold stock_barcode_rfid module): Done
  (module inactive) -- manifest/models/controllers/security all built
  and pushed before the pivot superseded the module
- Row 8 (2026-09-01, Source iData SDK): In Progress 50% -- SDK
  identified and integrated into the repo; on-device smoke test still
  outstanding, added as the explicit next action
- Row 21 (Discrepancies view): Superseded but replacement flagged
  Done -- UnresolvedScanStore.kt is the on-device equivalent, already
  built and pushed

Rows 3, 5, 6 (Docker, product field config, Android scaffold) and
everything from row 25 onward remain accurately Not Started -- no
work has actually been done on those yet.
</commit_message>
<xml_diff>
--- a/SEAN_TRACKER_MASTER.xlsx
+++ b/SEAN_TRACKER_MASTER.xlsx
@@ -72,7 +72,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,12 @@
         <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +156,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -228,6 +234,12 @@
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -563,42 +575,46 @@
       </c>
     </row>
     <row r="2" ht="45" customHeight="1" s="11">
-      <c r="A2" s="13" t="n">
+      <c r="A2" s="27" t="n">
         <v>46258</v>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>Confirm Phase 0 decisions log against locked constraints (T1UHF-only, Community, rfid.tag.mapping, Pilot/UAT scope).</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>Confirmed via chat: T1UHF-only, Community edition, Pilot/UAT scope, and (until the 2026-08-26 pivot) the rfid.tag.mapping design all cross-checked against rfid-odoo-roadmap-MASTER.docx Section 2 before any code was written.</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>Signed-off Phase 0 decisions matching rfid-odoo-roadmap-MASTER.docx Section 2.</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F2" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>See rfid-odoo-roadmap-MASTER.docx for phase context.</t>
-        </is>
-      </c>
-      <c r="J2" s="14" t="n"/>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L2" s="14" t="n"/>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" s="28" t="n"/>
+      <c r="H2" s="28" t="n"/>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>See rfid-odoo-roadmap-MASTER.docx for phase context.</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="n"/>
+      <c r="K2" s="28" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L2" s="28" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1" s="11">
       <c r="A3" s="15" t="n">
@@ -639,42 +655,46 @@
       <c r="L3" s="16" t="n"/>
     </row>
     <row r="4" ht="45" customHeight="1" s="11">
-      <c r="A4" s="13" t="n">
+      <c r="A4" s="19" t="n">
         <v>46260</v>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Scaffold stock_barcode_rfid Odoo module (manifest, models/, controllers/, views/, security/, tests/).</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Manifest, models/ (rfid.tag.mapping, stock.barcode.rfid.scan), controllers/ (POST /stock_barcode_rfid/scan), security/ir.model.access.csv all built and pushed. Module later marked inactive by the 2026-08-26 pivot -- code retained, not deleted.</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Empty module installs without errors.</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="14" t="n"/>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>See rfid-odoo-roadmap-MASTER.docx for phase context.</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="n"/>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="n"/>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Done (module inactive -- see 2026-08-26 addendum)</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="20" t="n"/>
+      <c r="H4" s="20" t="n"/>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>See rfid-odoo-roadmap-MASTER.docx for phase context.</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="n"/>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="n"/>
     </row>
     <row r="5" ht="45" customHeight="1" s="11">
       <c r="A5" s="15" t="n">
@@ -783,42 +803,46 @@
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" s="11">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="19" t="n">
         <v>46266</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Source and import the iData T1UHF SDK (.aar/.jar); resolve Gradle dependencies; smoke-test SDK init on the physical device.</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>UHFJar_V1.4.05.aar + native libs (libjni_rfid_driver.so, libserialportJni.so for arm64-v8a/armeabi-v7a) identified as the correct iData-branded SDK (of 3 IT-provided candidates) and committed into android/app/libs and jniLibs. Demo APK (UHFDemo_v1.2.534) provided for on-device sideload. Smoke test on the physical T1UHF unit not yet confirmed back.</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>SDK initializes; device responds to open()/powerOn()-equivalent call. CRITICAL PATH ITEM.</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>See rfid-odoo-roadmap-MASTER.docx for phase context.</t>
-        </is>
-      </c>
-      <c r="J8" s="14" t="n"/>
-      <c r="K8" s="14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L8" s="14" t="n"/>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="G8" s="20" t="n"/>
+      <c r="H8" s="20" t="n"/>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>Sideload UHFDemo_v1.2.534 APK onto the physical T1UHF and confirm scan/inventory works.</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="n"/>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L8" s="20" t="n"/>
     </row>
     <row r="9" ht="45" customHeight="1" s="11">
       <c r="A9" s="19" t="n">
@@ -1341,7 +1365,11 @@
           <t>Discrepancies view: list all stock.barcode.rfid.scan rows with status='unknown' for operator resolution (Ventor 'Discrepancies' pattern).</t>
         </is>
       </c>
-      <c r="C21" s="24" t="n"/>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>Replacement built: UnresolvedScanStore.kt (local SQLite) logs every EPC that fails to match, so operators can still review unresolved tags. This is the on-device equivalent of the original server-side Discrepancies view.</t>
+        </is>
+      </c>
       <c r="D21" s="24" t="inlineStr">
         <is>
           <t>View shows unresolved EPCs with product context where available.</t>
@@ -1349,11 +1377,11 @@
       </c>
       <c r="E21" s="24" t="inlineStr">
         <is>
-          <t>Superseded (see 2026-08-26 addendum)</t>
+          <t>Superseded -- replacement implemented (see 2026-08-26 addendum)</t>
         </is>
       </c>
       <c r="F21" s="24" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G21" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mark Android scaffold task In Progress (25%) per Desktop 1 confirmation
Vin confirmed RfidScannerApp2 work has started on Desktop 1, but exact
current state isn't confirmed and the real files aren't in this repo
yet -- this repo's android/ folder is still the unrelated older Kotlin
skeleton. Flagged as the explicit next action rather than marked Done
for work that hasn't been verified or merged here.
</commit_message>
<xml_diff>
--- a/SEAN_TRACKER_MASTER.xlsx
+++ b/SEAN_TRACKER_MASTER.xlsx
@@ -735,42 +735,50 @@
       <c r="L5" s="16" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1" s="11">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="19" t="n">
         <v>46262</v>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Scaffold Android project (Kotlin); package structure; Git branch strategy.</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Per Desktop 1: an Android app (RfidScannerApp2, Java, package com.manilainvestments.rfidscanner, using UHFManager/UM_MODULE) has started -- exact current state not yet confirmed against this repo.</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>Android project builds; repo structure matches monorepo convention.</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14" t="n"/>
-      <c r="H6" s="14" t="n"/>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>See rfid-odoo-roadmap-MASTER.docx for phase context.</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="n"/>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L6" s="14" t="n"/>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Real app lives in a separate session (Desktop 1), not yet merged into this repo. This repo's android/ folder is still the older, unrelated Kotlin skeleton (com.idataproject).</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="n"/>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>Confirm RfidScannerApp2’s current state with Vin and merge the real project files into this repo’s android/ folder.</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="n"/>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L6" s="20" t="n"/>
     </row>
     <row r="7" ht="19.5" customHeight="1" s="11">
       <c r="A7" s="17" t="n">

</xml_diff>

<commit_message>
Fill Supervisor/Remarks with technical review notes on completed work
Added genuine assessment for every row with actual progress (Done,
In Progress, or a superseded task whose replacement was built) --
code quality, real risks, what's still unverified. Left 'Pending' on
rows with no work done yet; nothing to assess there.

Notably flagged on row 21: Option 3 doesn't by itself satisfy the
never-drop-an-EPC success criterion -- UnresolvedScanStore exists but
isn't wired into any real scan loop yet.

Added a Tracker Guide note clarifying these are Claude's technical
review, not an official human supervisor sign-off -- the real OJT
supervisor should still review and countersign separately.
</commit_message>
<xml_diff>
--- a/SEAN_TRACKER_MASTER.xlsx
+++ b/SEAN_TRACKER_MASTER.xlsx
@@ -611,7 +611,7 @@
       <c r="J2" s="28" t="n"/>
       <c r="K2" s="28" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Adequate. Constraints were cross-checked against the roadmap before any code was written, which is the right order of operations -- low risk of rework from this step.</t>
         </is>
       </c>
       <c r="L2" s="28" t="n"/>
@@ -691,7 +691,7 @@
       <c r="J4" s="20" t="n"/>
       <c r="K4" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Technically clean at the time it was built (correct manifest, no Enterprise deps). Value is now moot since the module was superseded hours later -- not wasted effort, but a sign of how fast the direction changed this week.</t>
         </is>
       </c>
       <c r="L4" s="20" t="n"/>
@@ -775,7 +775,7 @@
       <c r="J6" s="20" t="n"/>
       <c r="K6" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Real gap: this work is happening in an un-synced separate session (Desktop 1). Until those files are merged here, this repo does not actually have a working Android scaffold. This is a coordination risk, not a technical one -- flag it as such.</t>
         </is>
       </c>
       <c r="L6" s="20" t="n"/>
@@ -847,7 +847,7 @@
       <c r="J8" s="20" t="n"/>
       <c r="K8" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>SDK selection was done properly -- cross-referenced 3 candidates against actual doc content instead of trusting filenames. But the step that actually matters (does it work on the real device) is still unconfirmed. Do not close this out until that smoke test comes back positive.</t>
         </is>
       </c>
       <c r="L8" s="20" t="n"/>
@@ -899,7 +899,11 @@
           <t>See rfid-odoo-roadmap-MASTER.docx Section 9 for full rationale.</t>
         </is>
       </c>
-      <c r="K9" s="20" t="n"/>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>Necessary and well-executed. Documenting an architecture reversal instead of silently overwriting the roadmap avoids confusion for whoever picks this up next.</t>
+        </is>
+      </c>
       <c r="L9" s="20" t="n"/>
     </row>
     <row r="10" ht="45" customHeight="1" s="11">
@@ -939,7 +943,7 @@
       <c r="J10" s="20" t="n"/>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Design was correct for its time (lot_id optional, EPC unique). Now inactive, but worth keeping -- if Option 3 runs into the unresolved-EPC problem during the pilot, this is a ready fallback.</t>
         </is>
       </c>
       <c r="L10" s="20" t="n"/>
@@ -981,7 +985,7 @@
       <c r="J11" s="20" t="n"/>
       <c r="K11" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>The stock.inventory -&gt; stock.location catch (Odoo 14+ removed that model) shows this was actually checked against the real Odoo 19 API, not written from memory. Good catch, now sitting unused.</t>
         </is>
       </c>
       <c r="L11" s="20" t="n"/>
@@ -1065,7 +1069,7 @@
       <c r="J13" s="20" t="n"/>
       <c r="K13" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Tests are written, not run -- there is no Docker/Odoo environment in this project yet. Treat 'Done' here as 'written', not 'passing'.</t>
         </is>
       </c>
       <c r="L13" s="20" t="n"/>
@@ -1107,7 +1111,7 @@
       <c r="J14" s="20" t="n"/>
       <c r="K14" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Endpoint is correctly built but is dead code under Option 3. No harm keeping it, but don't let it drift out of sync if anyone touches it later.</t>
         </is>
       </c>
       <c r="L14" s="20" t="n"/>
@@ -1149,7 +1153,7 @@
       <c r="J15" s="24" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L15" s="24" t="n"/>
@@ -1191,7 +1195,7 @@
       <c r="J16" s="24" t="n"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L16" s="24" t="n"/>
@@ -1233,7 +1237,7 @@
       <c r="J17" s="24" t="n"/>
       <c r="K17" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L17" s="24" t="n"/>
@@ -1275,7 +1279,7 @@
       <c r="J18" s="24" t="n"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L18" s="24" t="n"/>
@@ -1317,7 +1321,7 @@
       <c r="J19" s="24" t="n"/>
       <c r="K19" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L19" s="24" t="n"/>
@@ -1359,7 +1363,7 @@
       <c r="J20" s="24" t="n"/>
       <c r="K20" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L20" s="24" t="n"/>
@@ -1405,7 +1409,7 @@
       <c r="J21" s="24" t="n"/>
       <c r="K21" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>The most important remark on this sheet: Option 3 does not by itself guarantee the "never silently drop an EPC" success criterion. UnresolvedScanStore is built, but not yet called from any actual scan loop -- it is a solution sitting on a shelf until the real Android code wires it in.</t>
         </is>
       </c>
       <c r="L21" s="24" t="n"/>
@@ -1447,7 +1451,7 @@
       <c r="J22" s="24" t="n"/>
       <c r="K22" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L22" s="24" t="n"/>
@@ -1489,7 +1493,7 @@
       <c r="J23" s="24" t="n"/>
       <c r="K23" s="24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Correctly superseded, no code debt.</t>
         </is>
       </c>
       <c r="L23" s="24" t="n"/>
@@ -2317,7 +2321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="10" min="1" max="1"/>
@@ -2444,6 +2448,18 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Supervisor / Remarks column (as of 2026-08-26)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Entries filled in for rows with actual progress are Claude's own technical review of the work (code quality, real risks, what's still unverified) -- not an official human supervisor's sign-off. Your actual OJT supervisor should still review and countersign separately; do not submit this column as-is as their approval.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>